<commit_message>
Hotel data: about copy, no Cinta Costera
</commit_message>
<xml_diff>
--- a/data/hotel-page-data.xlsx
+++ b/data/hotel-page-data.xlsx
@@ -490,12 +490,8 @@
           <t>Golden Vacation and Travel - Hotel page data</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="2"/>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -3975,22 +3971,22 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Avenida Balboa, Panama Bay, Cinta Costera</t>
+          <t>Avenida Balboa, Panama Bay</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>Avenida Balboa, Cinta Costera, Panama Bay, the financial district</t>
+          <t>Avenida Balboa, Panama Bay, the financial district</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>The Financial District, Avenida Balboa, Cinta Costera</t>
+          <t>The Financial District, Avenida Balboa</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
-          <t>Multiplaza Pacific Mall, Old Panama, ATLAPA Convention Centre, Cinta Costera</t>
+          <t>Multiplaza Pacific Mall, Old Panama, ATLAPA Convention Centre</t>
         </is>
       </c>
       <c r="M23" s="6" t="inlineStr">
@@ -4035,7 +4031,7 @@
       </c>
       <c r="U23" s="6" t="inlineStr">
         <is>
-          <t>Calle 50, Marbella, Cinta Costera, Multiplaza Pacific</t>
+          <t>Calle 50, Marbella, Multiplaza Pacific</t>
         </is>
       </c>
       <c r="V23" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Hotel data: Deluxe Twin note removed
</commit_message>
<xml_diff>
--- a/data/hotel-page-data.xlsx
+++ b/data/hotel-page-data.xlsx
@@ -491,7 +491,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -14662,11 +14661,7 @@
           <t>2 beds 125x200</t>
         </is>
       </c>
-      <c r="G161" s="6" t="inlineStr">
-        <is>
-          <t>Code DLT. The adapted rooms sit in this category.</t>
-        </is>
-      </c>
+      <c r="G161" s="6" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="6" t="inlineStr">

</xml_diff>

<commit_message>
hotel sheet: Riu Playa Blanca Triple Room beds
</commit_message>
<xml_diff>
--- a/data/hotel-page-data.xlsx
+++ b/data/hotel-page-data.xlsx
@@ -15278,17 +15278,17 @@
       </c>
       <c r="E178" s="6" t="inlineStr">
         <is>
-          <t>On request</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F178" s="6" t="inlineStr">
         <is>
-          <t>On request</t>
+          <t>One king bed and one small double bed</t>
         </is>
       </c>
       <c r="G178" s="6" t="inlineStr">
         <is>
-          <t>Sofa bed. Code TBSB.</t>
+          <t>Code TBSB.</t>
         </is>
       </c>
     </row>

</xml_diff>